<commit_message>
gave up on kcfinder.  It wouldn't work because we can't store images in our file structure because of Docker.  Instead, we'll let them link to images stored elsewhere.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@195 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -1,21 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fmcgrath\Desktop\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="25725"/>
+  <workbookPr autoCompressPictures="0"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23055" windowHeight="9840"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23480" windowHeight="15860"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="140001" concurrentCalc="0"/>
   <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
+      <mx:ArchID Flags="2"/>
+    </ext>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
@@ -24,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
   <si>
     <t>Clickable glossed text doesn't work well in Sanskrit.  Should we display it like the old system?</t>
   </si>
@@ -123,6 +121,9 @@
   </si>
   <si>
     <t>L for me, XL for you</t>
+  </si>
+  <si>
+    <t>Autosave every 5 seconds</t>
   </si>
 </sst>
 </file>
@@ -246,7 +247,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
+        <a:latin typeface="Calibri Light"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -281,7 +282,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -458,7 +459,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -466,15 +467,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
   <cols>
-    <col min="1" max="1" width="88.5703125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="2"/>
+    <col min="1" max="1" width="88.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.1640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" s="5" customFormat="1">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
@@ -485,192 +486,274 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="18.75" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C3" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C4" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="C5" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C6" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C8" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="C9" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="28">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C10" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="C11" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="28">
       <c r="A12" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C12" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C13" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="C14" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="28">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="C15" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="17" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C16" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="28">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C18" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C19" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="28">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="C20" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
       <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C21" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C22" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
       <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C23" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
       <c r="A24" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>20</v>
       </c>
+      <c r="C24" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C27" s="2">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait"/>
+  <extLst>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
+      <mx:PLV Mode="0" OnePage="0" WScale="0"/>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
First pass at printable PDF.  It returns all lessons in one html doc.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@197 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -1,28 +1,33 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="25725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr autoCompressPictures="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fmcgrath\workspace\lrc-site\Documentation\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23480" windowHeight="15860"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23475" windowHeight="15855"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="140001" concurrentCalc="0"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
   <si>
     <t>Clickable glossed text doesn't work well in Sanskrit.  Should we display it like the old system?</t>
   </si>
@@ -124,6 +129,15 @@
   </si>
   <si>
     <t>Autosave every 5 seconds</t>
+  </si>
+  <si>
+    <t>Donate button</t>
+  </si>
+  <si>
+    <t>Google Analytics</t>
+  </si>
+  <si>
+    <t>?</t>
   </si>
 </sst>
 </file>
@@ -459,7 +473,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" xmlns="" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -467,15 +481,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.1640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" style="2"/>
+    <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1">
+    <row r="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>16</v>
       </c>
@@ -486,7 +500,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1">
+    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -497,7 +511,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1">
+    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -508,7 +522,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -519,7 +533,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
@@ -530,7 +544,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
@@ -541,7 +555,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>4</v>
       </c>
@@ -552,7 +566,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>5</v>
       </c>
@@ -563,7 +577,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>24</v>
       </c>
@@ -574,7 +588,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="28">
+    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
@@ -585,7 +599,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
@@ -596,7 +610,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="28">
+    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>25</v>
       </c>
@@ -607,7 +621,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>7</v>
       </c>
@@ -618,7 +632,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>8</v>
       </c>
@@ -629,7 +643,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="28">
+    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>9</v>
       </c>
@@ -640,7 +654,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>10</v>
       </c>
@@ -651,7 +665,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="28">
+    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -662,7 +676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:3">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>28</v>
       </c>
@@ -673,7 +687,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>29</v>
       </c>
@@ -684,7 +698,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="28">
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>30</v>
       </c>
@@ -695,7 +709,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>12</v>
       </c>
@@ -706,7 +720,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>13</v>
       </c>
@@ -717,7 +731,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>14</v>
       </c>
@@ -728,7 +742,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>15</v>
       </c>
@@ -739,12 +753,34 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C27" s="2">
         <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C28" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
On lesson page, warn if they try to leave before saving changes.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@201 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="38">
   <si>
     <t>Clickable glossed text doesn't work well in Sanskrit.  Should we display it like the old system?</t>
   </si>
@@ -128,9 +128,6 @@
     <t>L for me, XL for you</t>
   </si>
   <si>
-    <t>Autosave every 5 seconds</t>
-  </si>
-  <si>
     <t>Donate button</t>
   </si>
   <si>
@@ -138,6 +135,12 @@
   </si>
   <si>
     <t>?</t>
+  </si>
+  <si>
+    <t>Suloni's new design</t>
+  </si>
+  <si>
+    <t>DONE</t>
   </si>
 </sst>
 </file>
@@ -481,7 +484,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C27"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
@@ -502,288 +505,294 @@
     </row>
     <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="B2" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="2">
-        <v>2</v>
+      <c r="C2" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>19</v>
-      </c>
-      <c r="C5" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>21</v>
       </c>
       <c r="C6" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C8" s="2">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>4</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C10" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C11" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B12" s="6" t="s">
+      <c r="C12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B13" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>21</v>
-      </c>
       <c r="C13" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C14" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="C15" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>10</v>
+        <v>25</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C16" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C17" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="C18" s="2">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C19" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C20" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21" s="2">
         <v>4</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C20" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C21" s="2">
-        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C22" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="C23" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>20</v>
       </c>
       <c r="C24" s="2">
-        <v>2</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C25" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C27" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C28" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>36</v>
+      <c r="C27" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
+  <sortState ref="A2:C29">
+    <sortCondition ref="C1"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>
   <extLst>

</xml_diff>

<commit_message>
Warn if logon is about to expire.  Changed session length to 30 minutes.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@202 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
   <si>
     <t>Clickable glossed text doesn't work well in Sanskrit.  Should we display it like the old system?</t>
   </si>
@@ -521,8 +521,8 @@
       <c r="B3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C3" s="2">
-        <v>0</v>
+      <c r="C3" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
added previous and next buttons to lessons
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@204 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -12,7 +12,8 @@
     <workbookView xWindow="0" yWindow="0" windowWidth="23475" windowHeight="15855"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Francis" sheetId="1" r:id="rId1"/>
+    <sheet name="Todd" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="140001" concurrentCalc="0"/>
   <extLst>
@@ -27,13 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="38">
-  <si>
-    <t>Clickable glossed text doesn't work well in Sanskrit.  Should we display it like the old system?</t>
-  </si>
-  <si>
-    <t>Sort problems with ǣ and œ.  Some languages treat them as one character and others as two.</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="60">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -128,9 +123,6 @@
     <t>L for me, XL for you</t>
   </si>
   <si>
-    <t>Donate button</t>
-  </si>
-  <si>
     <t>Google Analytics</t>
   </si>
   <si>
@@ -141,13 +133,88 @@
   </si>
   <si>
     <t>DONE</t>
+  </si>
+  <si>
+    <t>DONE - Lesson editor only</t>
+  </si>
+  <si>
+    <t>DONE - Not on popups</t>
+  </si>
+  <si>
+    <t>Need to finalize design first</t>
+  </si>
+  <si>
+    <t>Coordindate design with Andre's redesign of center site</t>
+  </si>
+  <si>
+    <t>set up PROD.  Don't require VPN in PROD.  Load Prod DB.</t>
+  </si>
+  <si>
+    <t>waiting on Justin</t>
+  </si>
+  <si>
+    <t>set up location to store images</t>
+  </si>
+  <si>
+    <t>Sort problems with ǣ and œ.  Some languages treat them as one character and others as two. (hint: Look at Unicode Collation Algorithm. Perhaps just let them map characters like ǣ = ae.)</t>
+  </si>
+  <si>
+    <t>EIEOL Languages - review sort order</t>
+  </si>
+  <si>
+    <t>Mistakes with semi-colons in EIEOL</t>
+  </si>
+  <si>
+    <t>Help design a Unicode test page.  We will give them a bunch of text and a screenshot of what it should look like.</t>
+  </si>
+  <si>
+    <t>DOI - Digital Object Identifier - register with DOI sites.</t>
+  </si>
+  <si>
+    <t>Review links and toolbars with users</t>
+  </si>
+  <si>
+    <t>waiting on Andre</t>
+  </si>
+  <si>
+    <t>remove load controller, load views, references in routes.php and app/storage/data_load/</t>
+  </si>
+  <si>
+    <t>After implementation</t>
+  </si>
+  <si>
+    <t>Redirects - for each subfolder in http://www.utexas.edu/cola/centers/lrc/, redirect to appropriate location on new system</t>
+  </si>
+  <si>
+    <t>As part of release</t>
+  </si>
+  <si>
+    <t>Fix bugs, tweak UI</t>
+  </si>
+  <si>
+    <t>ONGOING</t>
+  </si>
+  <si>
+    <t>Donate button in new site</t>
+  </si>
+  <si>
+    <t>Add donate button to existing site</t>
+  </si>
+  <si>
+    <t>with Andre</t>
+  </si>
+  <si>
+    <t>Change Sanskrit lessons to not use clickable interface</t>
+  </si>
+  <si>
+    <t>TEST, TEST, TEST</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -159,6 +226,33 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B050"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -184,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -204,6 +298,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -484,309 +618,424 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.85546875" style="2"/>
+    <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="4" t="s">
+    </row>
+    <row r="2" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="C2" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C6" s="17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="9">
+        <v>0</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="9">
+        <v>0</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="9">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="9">
+        <v>0</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C11" s="2">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C7" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>10</v>
+        <v>47</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C12" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" s="10"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D16" s="10"/>
+    </row>
+    <row r="17" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="20"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="22" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C13" s="2">
+      <c r="B21" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C14" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C15" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C19" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C20" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C21" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C23" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C25" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="2">
+      <c r="C27" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C28" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C29" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C31" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C32" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C33" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C34" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C35" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C36" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B37" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B23" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C23" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="C37" s="2">
         <v>5</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C24" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B25" s="6" t="s">
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C25" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>35</v>
+      <c r="B38" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -794,11 +1043,49 @@
     <sortCondition ref="C1"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <extLst>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
       <mx:PLV Mode="0" OnePage="0" WScale="0"/>
     </ext>
   </extLst>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="102.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
First pass at authorizations
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@206 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -13,9 +13,10 @@
   </bookViews>
   <sheets>
     <sheet name="Francis" sheetId="1" r:id="rId1"/>
-    <sheet name="Todd" sheetId="2" r:id="rId2"/>
+    <sheet name="Done" sheetId="3" r:id="rId2"/>
+    <sheet name="Todd" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="140001" concurrentCalc="0"/>
+  <calcPr calcId="152511" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="63">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -150,9 +151,6 @@
     <t>set up PROD.  Don't require VPN in PROD.  Load Prod DB.</t>
   </si>
   <si>
-    <t>waiting on Justin</t>
-  </si>
-  <si>
     <t>set up location to store images</t>
   </si>
   <si>
@@ -208,6 +206,18 @@
   </si>
   <si>
     <t>TEST, TEST, TEST</t>
+  </si>
+  <si>
+    <t>Load new lessons that were started in the old system?</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Move content from Old site to center site.</t>
+  </si>
+  <si>
+    <t>In test and Prod, authorize Hans and Todd</t>
   </si>
 </sst>
 </file>
@@ -618,7 +628,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
@@ -627,7 +637,7 @@
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>14</v>
       </c>
@@ -638,222 +648,222 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="12" t="s">
+    <row r="2" spans="1:5" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="17">
+        <v>1</v>
+      </c>
+      <c r="D2" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="E2" s="18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="B3" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="13" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="12" t="s">
+      <c r="C3" s="17">
+        <v>0</v>
+      </c>
+      <c r="D3" s="18" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="9">
+        <v>0</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="9">
+        <v>0</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="13" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="12" t="s">
+      <c r="C7" s="2">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="B5" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="17">
+      <c r="C9" s="2">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="2">
+        <v>0</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D13" s="10"/>
+    </row>
+    <row r="14" spans="1:5" s="22" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="22" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B6" s="16" t="s">
+      <c r="B18" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="9">
-        <v>0</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="9">
-        <v>0</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" s="9">
-        <v>0</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B10" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="9">
-        <v>0</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="2">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C13" s="2">
-        <v>0</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C14" s="2">
-        <v>0</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D15" s="10"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D16" s="10"/>
-    </row>
-    <row r="17" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B17" s="20"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="22" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="C18" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C20" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C21" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C22" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>18</v>
@@ -862,53 +872,53 @@
         <v>2</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C24" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C25" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C26" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="C27" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>23</v>
+        <v>11</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>18</v>
@@ -917,124 +927,80 @@
         <v>3</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="C29" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>7</v>
+        <v>41</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C30" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C32" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31" s="6" t="s">
+      <c r="B33" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C31" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C32" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>19</v>
-      </c>
       <c r="C33" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C34" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C35" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C36" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C37" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="B38" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C39" s="2" t="s">
+      <c r="C35" s="2" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1054,7 +1020,125 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:D26"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="17"/>
+    </row>
+    <row r="8" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="15"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="17"/>
+    </row>
+    <row r="9" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="9"/>
+    </row>
+    <row r="11" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="9"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D14" s="10"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D15" s="10"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D18" s="10"/>
+    </row>
+    <row r="19" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="19"/>
+      <c r="B19" s="20"/>
+      <c r="C19" s="21"/>
+    </row>
+    <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="102.42578125" bestFit="1" customWidth="1"/>
@@ -1062,27 +1146,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>59</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added instructions for uploading images.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@207 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,14 +29,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
   <si>
-    <t>Authorizations.  Right now any admin user can update any lesson or lexicon.  Do we need to restrict users?</t>
-  </si>
-  <si>
     <t>When updating lessons - warn if the item has been updated since you loaded it.</t>
   </si>
   <si>
@@ -211,20 +208,20 @@
     <t>Load new lessons that were started in the old system?</t>
   </si>
   <si>
-    <t>In Progress</t>
-  </si>
-  <si>
     <t>Move content from Old site to center site.</t>
   </si>
   <si>
-    <t>In test and Prod, authorize Hans and Todd</t>
+    <t>Use EIDs instead of our own logons?</t>
+  </si>
+  <si>
+    <t>Authorizations.  Restrict users to certain series.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -260,13 +257,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF00B0F0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -288,7 +278,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -328,16 +318,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -628,7 +608,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:D34"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
@@ -637,192 +617,183 @@
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" s="18" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="17">
-        <v>1</v>
-      </c>
-      <c r="D2" s="18" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="18" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="17">
+    </row>
+    <row r="2" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" s="9">
         <v>0</v>
       </c>
-      <c r="D3" s="18" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D2" s="10" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>55</v>
+        <v>37</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" s="9">
         <v>0</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>53</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C6" s="9">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2">
         <v>0</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>54</v>
-      </c>
       <c r="B7" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="2">
         <v>0</v>
       </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D7" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="D8" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D11" s="10"/>
+    </row>
+    <row r="12" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="B12" s="16"/>
+      <c r="C12" s="17"/>
+      <c r="D12" s="18" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="2">
-        <v>0</v>
-      </c>
-      <c r="D9" s="10" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" s="2">
-        <v>0</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D13" s="10"/>
-    </row>
-    <row r="14" spans="1:5" s="22" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="B14" s="20"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="22" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="C15" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C18" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>22</v>
+        <v>7</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2">
         <v>2</v>
@@ -830,18 +801,18 @@
     </row>
     <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C20" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>17</v>
@@ -850,34 +821,34 @@
         <v>2</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C22" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C24" s="2">
         <v>3</v>
@@ -885,10 +856,10 @@
     </row>
     <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>23</v>
+        <v>6</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C25" s="2">
         <v>3</v>
@@ -896,54 +867,54 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C26" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C27" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C28" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C29" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C30" s="2">
         <v>4</v>
@@ -951,57 +922,40 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B31" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C31" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C32" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C33" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>29</v>
-      </c>
-      <c r="C34" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="B35" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>32</v>
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1031,79 +985,91 @@
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="11" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16"/>
-      <c r="C7" s="17"/>
-    </row>
-    <row r="8" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="16"/>
-      <c r="C8" s="17"/>
+      <c r="B8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="13">
+        <v>0</v>
+      </c>
     </row>
     <row r="9" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
@@ -1124,10 +1090,10 @@
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D18" s="10"/>
     </row>
-    <row r="19" spans="1:4" s="22" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="19"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="21"/>
+    <row r="19" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="15"/>
+      <c r="B19" s="16"/>
+      <c r="C19" s="17"/>
     </row>
     <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -1146,32 +1112,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added donate button to public pages.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@208 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23475" windowHeight="15855"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14955" windowHeight="7305"/>
   </bookViews>
   <sheets>
     <sheet name="Francis" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="59">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -139,9 +139,6 @@
     <t>DONE - Not on popups</t>
   </si>
   <si>
-    <t>Need to finalize design first</t>
-  </si>
-  <si>
     <t>Coordindate design with Andre's redesign of center site</t>
   </si>
   <si>
@@ -169,9 +166,6 @@
     <t>Review links and toolbars with users</t>
   </si>
   <si>
-    <t>waiting on Andre</t>
-  </si>
-  <si>
     <t>remove load controller, load views, references in routes.php and app/storage/data_load/</t>
   </si>
   <si>
@@ -184,12 +178,6 @@
     <t>As part of release</t>
   </si>
   <si>
-    <t>Fix bugs, tweak UI</t>
-  </si>
-  <si>
-    <t>ONGOING</t>
-  </si>
-  <si>
     <t>Donate button in new site</t>
   </si>
   <si>
@@ -205,9 +193,6 @@
     <t>TEST, TEST, TEST</t>
   </si>
   <si>
-    <t>Load new lessons that were started in the old system?</t>
-  </si>
-  <si>
     <t>Move content from Old site to center site.</t>
   </si>
   <si>
@@ -215,6 +200,12 @@
   </si>
   <si>
     <t>Authorizations.  Restrict users to certain series.</t>
+  </si>
+  <si>
+    <t>Add underlying form to gloss</t>
+  </si>
+  <si>
+    <t>wait till Andre finishes his redesign</t>
   </si>
 </sst>
 </file>
@@ -608,13 +599,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D34"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
@@ -628,34 +619,31 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" s="9">
-        <v>0</v>
-      </c>
-      <c r="D2" s="10" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
+    <row r="2" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>57</v>
+      </c>
+      <c r="B2" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="17">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="17" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B4" s="8" t="s">
         <v>18</v>
@@ -664,21 +652,18 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>46</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
-      </c>
-      <c r="D5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -686,18 +671,21 @@
         <v>45</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C6" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C7" s="2">
         <v>0</v>
@@ -706,61 +694,78 @@
         <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B8" s="6" t="s">
+    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C8" s="2">
-        <v>0</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D11" s="10"/>
-    </row>
-    <row r="12" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="15" t="s">
-        <v>51</v>
-      </c>
-      <c r="B12" s="16"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="18" t="s">
-        <v>52</v>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C15" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C16" s="2">
         <v>2</v>
@@ -768,65 +773,65 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C18" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C19" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="C20" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C21" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C22" s="2">
         <v>3</v>
@@ -834,128 +839,73 @@
     </row>
     <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>22</v>
+        <v>39</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C23" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="2">
         <v>4</v>
       </c>
-      <c r="B24" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C24" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>6</v>
+        <v>26</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C25" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C26" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C28" s="2">
-        <v>4</v>
+        <v>31</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C29" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C30" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C31" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C32" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1029,7 +979,7 @@
     </row>
     <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>16</v>
@@ -1040,7 +990,7 @@
     </row>
     <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>16</v>
@@ -1051,7 +1001,7 @@
     </row>
     <row r="7" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>18</v>
@@ -1062,7 +1012,7 @@
     </row>
     <row r="8" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>16</v>
@@ -1071,10 +1021,30 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="9"/>
+    <row r="9" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="13">
+        <v>0</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="13">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
@@ -1112,32 +1082,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
more changes to google analytics.  Put in external file and added to frozen node scripts.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@211 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="60">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -206,6 +206,9 @@
   </si>
   <si>
     <t>wait till Andre finishes his redesign</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> M</t>
   </si>
 </sst>
 </file>
@@ -599,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
@@ -630,128 +633,128 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B3" s="16" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="17" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="3" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B3" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="9">
+      <c r="C3" s="9">
         <v>0</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D3" s="10" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D5" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C6" s="2">
         <v>0</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" s="6" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2">
-        <v>0</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="C10" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C11" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C12" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>17</v>
@@ -762,54 +765,54 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B16" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="C16" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C18" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C20" s="2">
         <v>3</v>
@@ -817,32 +820,32 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C21" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>11</v>
+        <v>39</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="C22" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C23" s="2">
         <v>4</v>
@@ -850,10 +853,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C24" s="2">
         <v>4</v>
@@ -861,50 +864,39 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C25" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C26" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C27" s="2">
-        <v>5</v>
+        <v>31</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
         <v>55</v>
       </c>
     </row>
@@ -1046,10 +1038,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="9"/>
+    <row r="11" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="C11" s="13"/>
+      <c r="D11" s="14" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" s="10"/>

</xml_diff>

<commit_message>
extracted common code from layout and printable header layout into layout header.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@212 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="60">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -124,9 +124,6 @@
     <t>Google Analytics</t>
   </si>
   <si>
-    <t>?</t>
-  </si>
-  <si>
     <t>Suloni's new design</t>
   </si>
   <si>
@@ -209,6 +206,9 @@
   </si>
   <si>
     <t xml:space="preserve"> M</t>
+  </si>
+  <si>
+    <t>Copy a series</t>
   </si>
 </sst>
 </file>
@@ -602,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
@@ -624,7 +624,7 @@
     </row>
     <row r="2" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B2" s="16" t="s">
         <v>16</v>
@@ -635,7 +635,7 @@
     </row>
     <row r="3" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B3" s="8" t="s">
         <v>18</v>
@@ -644,12 +644,12 @@
         <v>0</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>18</v>
@@ -660,7 +660,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>16</v>
@@ -669,12 +669,12 @@
         <v>0</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>18</v>
@@ -683,7 +683,7 @@
         <v>0</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -831,7 +831,7 @@
     </row>
     <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>18</v>
@@ -886,18 +886,26 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -944,7 +952,7 @@
         <v>16</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -955,7 +963,7 @@
         <v>16</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -966,34 +974,34 @@
         <v>16</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>18</v>
@@ -1004,7 +1012,7 @@
     </row>
     <row r="8" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>16</v>
@@ -1015,7 +1023,7 @@
     </row>
     <row r="9" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>18</v>
@@ -1024,12 +1032,12 @@
         <v>0</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>16</v>
@@ -1043,11 +1051,11 @@
         <v>30</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -1081,32 +1089,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
-	Added underlying form field to gloss.  Added to lesson editor and the build gloss function in its model
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@213 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -602,7 +602,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
@@ -622,128 +622,128 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="B2" s="16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="17">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+    <row r="2" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="B2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C3" s="9">
+      <c r="C2" s="9">
         <v>0</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D2" s="10" t="s">
         <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D4" s="10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2">
         <v>0</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B6" s="6" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" s="2">
-        <v>0</v>
-      </c>
-      <c r="D6" s="10" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>17</v>
-      </c>
       <c r="C9" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>1</v>
+        <v>21</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C10" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C11" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>23</v>
+        <v>7</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C12" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>17</v>
@@ -754,54 +754,54 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="B15" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C15" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" s="6" t="s">
         <v>17</v>
-      </c>
-      <c r="C15" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>18</v>
       </c>
       <c r="C16" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="C18" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
@@ -809,32 +809,32 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C20" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>11</v>
+        <v>38</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="C21" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C22" s="2">
         <v>4</v>
@@ -842,10 +842,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C23" s="2">
         <v>4</v>
@@ -853,58 +853,47 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C24" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>2</v>
+        <v>27</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="C25" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C26" s="2">
-        <v>5</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>31</v>
+        <v>54</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B29" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1058,6 +1047,17 @@
         <v>50</v>
       </c>
     </row>
+    <row r="12" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="13">
+        <v>-1</v>
+      </c>
+    </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" s="10"/>
     </row>

</xml_diff>

<commit_message>
Created Rest function to return list of series for mobile testing
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@215 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="61">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -136,9 +136,6 @@
     <t>DONE - Not on popups</t>
   </si>
   <si>
-    <t>Coordindate design with Andre's redesign of center site</t>
-  </si>
-  <si>
     <t>set up PROD.  Don't require VPN in PROD.  Load Prod DB.</t>
   </si>
   <si>
@@ -209,6 +206,12 @@
   </si>
   <si>
     <t>Copy a series</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Make site look better on phones and ipads </t>
+  </si>
+  <si>
+    <t>Coordindate design with Andre's redesign of center site, fix mobile menu.</t>
   </si>
 </sst>
 </file>
@@ -602,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D29"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
@@ -624,7 +627,7 @@
     </row>
     <row r="2" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>35</v>
+        <v>60</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>18</v>
@@ -633,12 +636,12 @@
         <v>0</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>18</v>
@@ -649,7 +652,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>16</v>
@@ -658,12 +661,12 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>18</v>
@@ -672,7 +675,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -820,7 +823,7 @@
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>18</v>
@@ -883,7 +886,7 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>17</v>
@@ -891,9 +894,17 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B28" s="6" t="s">
+      <c r="B29" s="6" t="s">
         <v>18</v>
       </c>
     </row>
@@ -968,7 +979,7 @@
     </row>
     <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>16</v>
@@ -979,7 +990,7 @@
     </row>
     <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>16</v>
@@ -990,7 +1001,7 @@
     </row>
     <row r="7" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>18</v>
@@ -1001,7 +1012,7 @@
     </row>
     <row r="8" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>16</v>
@@ -1012,7 +1023,7 @@
     </row>
     <row r="9" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>18</v>
@@ -1021,12 +1032,12 @@
         <v>0</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>16</v>
@@ -1040,16 +1051,16 @@
         <v>30</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>16</v>
@@ -1089,32 +1100,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed bug in Gloss filtered list. Made bootstrap modals work better when opening more than one.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@221 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="72">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -94,15 +94,9 @@
     <t>XL</t>
   </si>
   <si>
-    <t>Add version control to the lessons so writers can track and revert changes.</t>
-  </si>
-  <si>
     <t>On lesson page, Reorder things by dragging.  Right now things can be reordered by typing a new number and refreshing the page.</t>
   </si>
   <si>
-    <t>On lesson page, save changes, and preview them without publishing. We would have to have versioning in place first.</t>
-  </si>
-  <si>
     <t>??</t>
   </si>
   <si>
@@ -218,6 +212,39 @@
   </si>
   <si>
     <t>Remove &lt;&gt; from headwords</t>
+  </si>
+  <si>
+    <t>When creating a new series, it's hard to remember what number to choose for the series order and the menu order, as well as what the format of the expanded title should be (it's not often that one creates an entire series).  So it might be helpful for the Create Series page to still list the existing series... if not the whole table, at least some summary data to help guide choices of ordering and naming.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> in Firefox and IE.</t>
+  </si>
+  <si>
+    <t>Delete Lesson button</t>
+  </si>
+  <si>
+    <t>Language Editor, rename edit button save.</t>
+  </si>
+  <si>
+    <t>Logging in by going to the login page directly instead of admin results in an error</t>
+  </si>
+  <si>
+    <t>In lesson editor, need a way of flagging glosses and textareas that have errors and add comment so another admin can fix</t>
+  </si>
+  <si>
+    <t>Programmatically split tables that are actually 2 tables so they display better on mobile devices</t>
+  </si>
+  <si>
+    <t>Add version control to the lessons so writers can track and revert changes.  An easier option of size (M) would be to add a copy feature.</t>
+  </si>
+  <si>
+    <t>On lesson page, save changes, and preview them without publishing. We would have to have versioning in place first.  Again, a copy feature would be easier.</t>
+  </si>
+  <si>
+    <t>Instead of loading images and movies to a different server, incoorporate Resource Space.</t>
+  </si>
+  <si>
+    <t>User pages have 2 scrollbars in IE an Firefox which makes scrolling weird.</t>
   </si>
 </sst>
 </file>
@@ -281,7 +308,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -331,6 +358,15 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -611,10 +647,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="88.42578125" style="19" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
@@ -633,7 +669,7 @@
     </row>
     <row r="2" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B2" s="8" t="s">
         <v>18</v>
@@ -642,12 +678,12 @@
         <v>0</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>42</v>
+      <c r="A3" s="19" t="s">
+        <v>40</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>18</v>
@@ -657,8 +693,8 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="1" t="s">
-        <v>43</v>
+      <c r="A4" s="19" t="s">
+        <v>41</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>16</v>
@@ -667,12 +703,12 @@
         <v>0</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
-        <v>45</v>
+      <c r="A5" s="19" t="s">
+        <v>43</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>18</v>
@@ -681,19 +717,19 @@
         <v>0</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
-        <v>61</v>
+      <c r="A6" s="19" t="s">
+        <v>59</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="19" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="6" t="s">
@@ -704,7 +740,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="19" t="s">
         <v>1</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -714,9 +750,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
-        <v>21</v>
+    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>68</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>20</v>
@@ -726,8 +762,8 @@
       </c>
     </row>
     <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>23</v>
+      <c r="A11" s="19" t="s">
+        <v>69</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>17</v>
@@ -737,7 +773,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="19" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -748,7 +784,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="19" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -759,7 +795,7 @@
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="19" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -770,7 +806,7 @@
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="1" t="s">
+      <c r="A15" s="19" t="s">
         <v>0</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -781,8 +817,8 @@
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>22</v>
+      <c r="A16" s="19" t="s">
+        <v>21</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>17</v>
@@ -792,7 +828,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
+      <c r="A17" s="19" t="s">
         <v>4</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -803,18 +839,18 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="1" t="s">
+      <c r="A18" s="19" t="s">
         <v>6</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C18" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="1" t="s">
+      <c r="A19" s="19" t="s">
         <v>10</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -825,19 +861,19 @@
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="19" t="s">
         <v>11</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C20" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>37</v>
+      <c r="A21" s="19" t="s">
+        <v>35</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>18</v>
@@ -847,7 +883,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
+      <c r="A22" s="19" t="s">
         <v>19</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -858,8 +894,8 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>26</v>
+      <c r="A23" s="19" t="s">
+        <v>24</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>17</v>
@@ -869,7 +905,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
+      <c r="A24" s="19" t="s">
         <v>2</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -880,54 +916,111 @@
       </c>
     </row>
     <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>27</v>
+      <c r="A25" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C25" s="2">
         <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>31</v>
+      <c r="A26" s="19" t="s">
+        <v>29</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>53</v>
+      <c r="A27" s="19" t="s">
+        <v>51</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>58</v>
+      <c r="A28" s="19" t="s">
+        <v>56</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>59</v>
+      <c r="A29" s="19" t="s">
+        <v>57</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>62</v>
+      <c r="A30" s="19" t="s">
+        <v>60</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A31" s="20" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="21" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="19" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="19" t="s">
+        <v>64</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A37" s="19" t="s">
+        <v>66</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="19" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -974,18 +1067,18 @@
         <v>16</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B3" s="12" t="s">
         <v>16</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
@@ -996,34 +1089,34 @@
         <v>16</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B5" s="12" t="s">
         <v>16</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B6" s="12" t="s">
         <v>16</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B7" s="12" t="s">
         <v>18</v>
@@ -1034,7 +1127,7 @@
     </row>
     <row r="8" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B8" s="12" t="s">
         <v>16</v>
@@ -1045,7 +1138,7 @@
     </row>
     <row r="9" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="12" t="s">
         <v>18</v>
@@ -1054,12 +1147,12 @@
         <v>0</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B10" s="12" t="s">
         <v>16</v>
@@ -1070,19 +1163,19 @@
     </row>
     <row r="11" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>16</v>
@@ -1122,32 +1215,32 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adjusted margin's of printable version
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@222 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="79">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -43,9 +43,6 @@
     <t>On lesson page, warn if they try to leave without saving something</t>
   </si>
   <si>
-    <t>On lesson page, delete an element from a gloss.</t>
-  </si>
-  <si>
     <t>EIEOL public pages  - next and prev buttons to go to other lessons.</t>
   </si>
   <si>
@@ -64,9 +61,6 @@
     <t>On lessons page, use high charts to graph 5 most used nouns and verbs</t>
   </si>
   <si>
-    <t>EIEOL - attach parts of speech to languages</t>
-  </si>
-  <si>
     <t>Link from Lexicon reflex to gloss</t>
   </si>
   <si>
@@ -112,9 +106,6 @@
     <t>L or XL</t>
   </si>
   <si>
-    <t>L for me, XL for you</t>
-  </si>
-  <si>
     <t>Google Analytics</t>
   </si>
   <si>
@@ -145,9 +136,6 @@
     <t>Mistakes with semi-colons in EIEOL</t>
   </si>
   <si>
-    <t>Help design a Unicode test page.  We will give them a bunch of text and a screenshot of what it should look like.</t>
-  </si>
-  <si>
     <t>DOI - Digital Object Identifier - register with DOI sites.</t>
   </si>
   <si>
@@ -217,21 +205,12 @@
     <t>When creating a new series, it's hard to remember what number to choose for the series order and the menu order, as well as what the format of the expanded title should be (it's not often that one creates an entire series).  So it might be helpful for the Create Series page to still list the existing series... if not the whole table, at least some summary data to help guide choices of ordering and naming.</t>
   </si>
   <si>
-    <t xml:space="preserve"> in Firefox and IE.</t>
-  </si>
-  <si>
     <t>Delete Lesson button</t>
   </si>
   <si>
-    <t>Language Editor, rename edit button save.</t>
-  </si>
-  <si>
     <t>Logging in by going to the login page directly instead of admin results in an error</t>
   </si>
   <si>
-    <t>In lesson editor, need a way of flagging glosses and textareas that have errors and add comment so another admin can fix</t>
-  </si>
-  <si>
     <t>Programmatically split tables that are actually 2 tables so they display better on mobile devices</t>
   </si>
   <si>
@@ -245,6 +224,48 @@
   </si>
   <si>
     <t>User pages have 2 scrollbars in IE an Firefox which makes scrolling weird.</t>
+  </si>
+  <si>
+    <t>The Rigveda and other IE Texts</t>
+  </si>
+  <si>
+    <t>On lesson editor, delete an element from a gloss.</t>
+  </si>
+  <si>
+    <t>Language Editor, rename "edit" button "save".</t>
+  </si>
+  <si>
+    <t>In lesson editor, need a way of flagging glosses and textareas that have mistakes and add comment so another admin can fix.  Admin comments (only admin can edit) Author comments.</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the editor, add links to instructional pages that Todd will create </t>
+  </si>
+  <si>
+    <t>XS</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>Design a Unicode test page.  Give them a bunch of text and a screenshot of what it should look like.</t>
+  </si>
+  <si>
+    <t>Decide what links to put in the menus on the new LRC site</t>
+  </si>
+  <si>
+    <t>Decide where to put links to the new LRC site on the center site</t>
+  </si>
+  <si>
+    <t>EIEOL - attach parts of speech and analysis to languages - use features file to load new one.  Sweep glosses to use new ones, change language editor, change pulldowns in gloss editor.  Add comment box to each pos and analysis.  Remove old POS and analysis editors</t>
   </si>
 </sst>
 </file>
@@ -308,7 +329,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -365,8 +386,12 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,10 +672,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.42578125" style="19" customWidth="1"/>
+    <col min="1" max="1" width="89.28515625" style="19" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
@@ -658,337 +683,331 @@
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="B2" s="8" t="s">
+    </row>
+    <row r="2" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="19" t="s">
+        <v>68</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A4" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C4" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="19" t="s">
+        <v>55</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="9">
         <v>0</v>
       </c>
-      <c r="D2" s="10" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
+      <c r="D7" s="10" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="22">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="19" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="22">
+        <v>0</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>40</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" s="2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
-        <v>41</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="2">
-        <v>0</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C5" s="2">
-        <v>0</v>
-      </c>
-      <c r="D5" s="10" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
-        <v>59</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C8" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C10" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
-        <v>69</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="2">
-        <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="19" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="19" t="s">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="19" t="s">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="B15" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="19" t="s">
-        <v>21</v>
+        <v>62</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C16" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="19" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C17" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="C18" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>27</v>
+        <v>15</v>
       </c>
       <c r="C20" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="19" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C21" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C22" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C23" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
-        <v>2</v>
-      </c>
-      <c r="B24" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C24" s="2">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C25" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
+      </c>
+      <c r="C26" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
+      </c>
+      <c r="C27" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>56</v>
+        <v>2</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="C28" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A29" s="19" t="s">
-        <v>57</v>
+        <v>23</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>18</v>
+        <v>24</v>
+      </c>
+      <c r="C29" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A31" s="20" t="s">
-        <v>61</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>15</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="21" t="s">
-        <v>62</v>
+      <c r="A32" s="19" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="19" t="s">
-        <v>71</v>
+        <v>53</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
-        <v>64</v>
+        <v>56</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A35" s="20" t="s">
+        <v>57</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>16</v>
@@ -996,18 +1015,18 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="37" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="19" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
@@ -1015,12 +1034,47 @@
         <v>67</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="19" t="s">
-        <v>70</v>
+        <v>59</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="19" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="19" t="s">
+        <v>65</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1050,13 +1104,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="4" t="s">
         <v>13</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1064,62 +1118,62 @@
         <v>3</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="11" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="11" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="11" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C7" s="13">
         <v>1</v>
@@ -1127,10 +1181,10 @@
     </row>
     <row r="8" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C8" s="13">
         <v>0</v>
@@ -1138,24 +1192,24 @@
     </row>
     <row r="9" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C9" s="13">
         <v>0</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C10" s="13">
         <v>0</v>
@@ -1163,22 +1217,22 @@
     </row>
     <row r="11" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="C11" s="13"/>
       <c r="D11" s="14" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="13">
         <v>-1</v>
@@ -1207,7 +1261,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="102.42578125" bestFit="1" customWidth="1"/>
@@ -1215,32 +1269,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>38</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added CK Editor to Glossed Texts
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@223 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="83">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -238,9 +238,6 @@
     <t>In lesson editor, need a way of flagging glosses and textareas that have mistakes and add comment so another admin can fix.  Admin comments (only admin can edit) Author comments.</t>
   </si>
   <si>
-    <t>A1</t>
-  </si>
-  <si>
     <t>A2</t>
   </si>
   <si>
@@ -266,6 +263,21 @@
   </si>
   <si>
     <t>EIEOL - attach parts of speech and analysis to languages - use features file to load new one.  Sweep glosses to use new ones, change language editor, change pulldowns in gloss editor.  Add comment box to each pos and analysis.  Remove old POS and analysis editors</t>
+  </si>
+  <si>
+    <t>umlauts are adding a space after the letter in some browsers.  See https://lrc.la.utexas.edu/eieol_lesson/7?id=929 - Grammars/2nd paragraph/1st word.  Browser specific?</t>
+  </si>
+  <si>
+    <t>Link to Bibliography in side bar, under lesson resources</t>
+  </si>
+  <si>
+    <t>Foreign Words that are marked like "&lt;span lang="non" class="Unicode"&gt;víkingr&lt;/span&gt;" need to stand out</t>
+  </si>
+  <si>
+    <t>Add marking foreign words as a push-button feature in CKEditor.  Does this tie nito the CKEditor item below?</t>
+  </si>
+  <si>
+    <t>Done</t>
   </si>
 </sst>
 </file>
@@ -329,7 +341,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -392,6 +404,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -672,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D48"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="89.28515625" style="19" customWidth="1"/>
@@ -692,15 +707,15 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="19" t="s">
+    <row r="2" spans="1:4" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>69</v>
+      <c r="B2" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -711,18 +726,18 @@
         <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>18</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -733,348 +748,368 @@
         <v>14</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="19" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="19" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="19" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A9" s="19" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="B7" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="9">
+      <c r="B12" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="9">
         <v>0</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D12" s="10" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
+    <row r="13" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="22">
+      <c r="B13" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="22">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
+    <row r="14" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="B9" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" s="22">
+      <c r="B14" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="22">
         <v>0</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D14" s="10" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="19" t="s">
+    <row r="15" spans="1:4" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="22">
+      <c r="B15" s="21" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="22">
         <v>0</v>
       </c>
-      <c r="D10" s="10" t="s">
+      <c r="D15" s="10" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+    <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="24" t="s">
         <v>7</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
-        <v>62</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="19" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="19" t="s">
-        <v>10</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C18" s="2">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="19" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>16</v>
       </c>
       <c r="C19" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="19" t="s">
-        <v>19</v>
+        <v>61</v>
       </c>
       <c r="B20" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="19" t="s">
+        <v>62</v>
+      </c>
+      <c r="B21" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C20" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>16</v>
-      </c>
       <c r="C21" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="19" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C22" s="2">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="19" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C23" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="19" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="19" t="s">
-        <v>32</v>
+        <v>19</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C25" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="19" t="s">
-        <v>17</v>
+        <v>66</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C26" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="19" t="s">
-        <v>22</v>
+        <v>5</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C27" s="2">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="19" t="s">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C28" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A29" s="19" t="s">
-        <v>23</v>
-      </c>
-      <c r="B29" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C29" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A30" s="19" t="s">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>16</v>
+      </c>
+      <c r="C30" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="19" t="s">
-        <v>47</v>
+        <v>17</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="C31" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C32" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="19" t="s">
+        <v>2</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C33" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A34" s="19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="19" t="s">
+        <v>26</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="19" t="s">
+        <v>47</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B32" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="19" t="s">
+      <c r="B37" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="B33" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
+      <c r="B38" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="B34" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A35" s="20" t="s">
+      <c r="B39" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="75" x14ac:dyDescent="0.25">
+      <c r="A40" s="20" t="s">
         <v>57</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
+      <c r="B40" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
+      <c r="B41" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B37" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="19" t="s">
+      <c r="B42" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="B38" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="19" t="s">
+      <c r="B43" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="B39" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="19" t="s">
+      <c r="B44" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B45" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="19" t="s">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B46" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="19" t="s">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B47" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="19" t="s">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="B48" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1279,7 +1314,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -1299,12 +1334,12 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed datatables on lang reflex page
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@224 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="82">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -250,9 +250,6 @@
     <t>XS</t>
   </si>
   <si>
-    <t>A4</t>
-  </si>
-  <si>
     <t>Design a Unicode test page.  Give them a bunch of text and a screenshot of what it should look like.</t>
   </si>
   <si>
@@ -274,10 +271,10 @@
     <t>Foreign Words that are marked like "&lt;span lang="non" class="Unicode"&gt;víkingr&lt;/span&gt;" need to stand out</t>
   </si>
   <si>
-    <t>Add marking foreign words as a push-button feature in CKEditor.  Does this tie nito the CKEditor item below?</t>
-  </si>
-  <si>
     <t>Done</t>
+  </si>
+  <si>
+    <t>Add marking foreign words as a push-button feature in CKEditor.  Does this tie ito the CKEditor item below?</t>
   </si>
 </sst>
 </file>
@@ -715,7 +712,7 @@
         <v>14</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -731,7 +728,7 @@
     </row>
     <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B4" s="6" t="s">
         <v>18</v>
@@ -740,30 +737,30 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="19" t="s">
+    <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>73</v>
+      <c r="B5" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="19" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="19" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="19" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
@@ -1314,7 +1311,7 @@
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -1334,12 +1331,12 @@
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added bibliography to menu
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@227 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="83">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -274,14 +274,17 @@
     <t>Done</t>
   </si>
   <si>
-    <t>Add marking foreign words as a push-button feature in CKEditor.  Does this tie ito the CKEditor item below?</t>
+    <t>early lesson series often had the bibliography as a section in the 10th lesson.  Later lessons have a bibliography that is essentially a separate page.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add marking foreign words as a push-button feature in CKEditor. </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -317,6 +320,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF00B050"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -338,7 +347,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -358,15 +367,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -404,6 +404,7 @@
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -684,10 +685,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="89.28515625" style="19" customWidth="1"/>
+    <col min="1" max="1" width="89.28515625" style="16" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
@@ -704,203 +705,205 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="14" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="13" t="s">
+    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A2" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="A3" s="16" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="19" t="s">
-        <v>68</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A4" s="19" t="s">
-        <v>76</v>
-      </c>
-      <c r="B4" s="6" t="s">
+      <c r="D4" s="22" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="16" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="16" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="21"/>
+    </row>
+    <row r="10" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="19">
+        <v>0</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B12" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="19">
+        <v>0</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A6" s="19" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="19" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A9" s="19" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="B12" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="9">
-        <v>0</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B13" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" s="23" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" s="22">
-        <v>0</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" s="23" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
-        <v>39</v>
-      </c>
-      <c r="B15" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="C15" s="22">
-        <v>0</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>40</v>
+      <c r="C17" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="24" t="s">
-        <v>7</v>
+      <c r="A18" s="16" t="s">
+        <v>62</v>
       </c>
       <c r="B18" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C18" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="19" t="s">
-        <v>1</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="16" t="s">
+        <v>8</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C19" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="19" t="s">
-        <v>61</v>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="16" t="s">
+        <v>10</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C20" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A21" s="19" t="s">
-        <v>62</v>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="16" t="s">
+        <v>0</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C21" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="19" t="s">
-        <v>8</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
+        <v>19</v>
       </c>
       <c r="B22" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C22" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="19" t="s">
-        <v>10</v>
+      <c r="A23" s="16" t="s">
+        <v>66</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C23" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="19" t="s">
-        <v>0</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="16" t="s">
+        <v>5</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="C24" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="19" t="s">
-        <v>19</v>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="16" t="s">
+        <v>9</v>
       </c>
       <c r="B25" s="6" t="s">
         <v>15</v>
@@ -909,203 +912,170 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="19" t="s">
-        <v>66</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C26" s="2">
-        <v>3</v>
-      </c>
-    </row>
     <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="19" t="s">
+      <c r="A27" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C27" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C30" s="2">
         <v>5</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C27" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="19" t="s">
-        <v>9</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C28" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="19" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="19" t="s">
-        <v>17</v>
+    </row>
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
+        <v>23</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="C31" s="2">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="19" t="s">
-        <v>22</v>
+      <c r="A32" s="16" t="s">
+        <v>26</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C32" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="19" t="s">
-        <v>2</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="16" t="s">
+        <v>47</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C33" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="19" t="s">
-        <v>23</v>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="16" t="s">
+        <v>52</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C34" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="19" t="s">
-        <v>26</v>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="16" t="s">
+        <v>53</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="19" t="s">
-        <v>47</v>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="16" t="s">
+        <v>56</v>
       </c>
       <c r="B36" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A37" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="B42" s="6" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="19" t="s">
-        <v>52</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="19" t="s">
-        <v>53</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="19" t="s">
-        <v>56</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" ht="75" x14ac:dyDescent="0.25">
-      <c r="A40" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="19" t="s">
-        <v>64</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="19" t="s">
-        <v>67</v>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="16" t="s">
+        <v>63</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="19" t="s">
-        <v>59</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="16" t="s">
+        <v>65</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="19" t="s">
-        <v>60</v>
+        <v>18</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="16" t="s">
+        <v>71</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="19" t="s">
-        <v>65</v>
-      </c>
-      <c r="B47" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="B48" s="6" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1145,144 +1115,185 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+    <row r="2" spans="1:4" s="11" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" s="13" t="s">
+      <c r="B2" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="14" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="11" t="s">
+    <row r="3" spans="1:4" s="11" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="B3" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="13" t="s">
+      <c r="B3" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="11" t="s">
+    <row r="4" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="13" t="s">
+      <c r="B4" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="11" t="s">
+    <row r="5" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" s="13" t="s">
+      <c r="B5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="11" t="s">
+    <row r="6" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="13" t="s">
+      <c r="B6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="11" t="s">
+    <row r="7" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="13">
+      <c r="B7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="10">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="11" t="s">
+    <row r="8" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="13">
+      <c r="B8" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="10">
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="11" t="s">
+    <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C9" s="13">
+      <c r="B9" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="10">
         <v>0</v>
       </c>
-      <c r="D9" s="14" t="s">
+      <c r="D9" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="11" t="s">
+    <row r="10" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="13">
+      <c r="B10" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="10">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="11" t="s">
+    <row r="11" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="14" t="s">
+      <c r="C11" s="10"/>
+      <c r="D11" s="11" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="14" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="11" t="s">
+    <row r="12" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="13">
+      <c r="B12" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="10">
         <v>-1</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D14" s="10"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D15" s="10"/>
+    <row r="13" spans="1:4" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C16" s="10">
+        <v>0</v>
+      </c>
+      <c r="D16" s="11" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="10"/>
-    </row>
-    <row r="19" spans="1:4" s="18" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16"/>
-      <c r="C19" s="17"/>
+      <c r="D18" s="7"/>
+    </row>
+    <row r="19" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="12"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="14"/>
     </row>
     <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>

<commit_message>
Added italics to different language css
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@229 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -278,6 +278,9 @@
   </si>
   <si>
     <t xml:space="preserve">Add marking foreign words as a push-button feature in CKEditor. </t>
+  </si>
+  <si>
+    <t>Fixed bullet formatting</t>
   </si>
 </sst>
 </file>
@@ -347,7 +350,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -401,9 +404,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -685,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D46"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="89.28515625" style="16" customWidth="1"/>
@@ -735,7 +735,7 @@
       <c r="C4" s="10" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>81</v>
       </c>
     </row>
@@ -760,65 +760,65 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="21"/>
-    </row>
-    <row r="10" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10" s="19">
-        <v>0</v>
-      </c>
+    <row r="8" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="10" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="10"/>
     </row>
     <row r="11" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C11" s="19">
         <v>0</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="19">
         <v>0</v>
       </c>
       <c r="D12" s="7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="19">
+        <v>0</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>61</v>
-      </c>
       <c r="B17" s="6" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C17" s="2">
         <v>2</v>
@@ -826,18 +826,18 @@
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C18" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
-        <v>8</v>
+        <v>62</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>15</v>
@@ -846,9 +846,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>15</v>
@@ -859,76 +859,76 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C21" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
-        <v>19</v>
-      </c>
       <c r="B22" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C22" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C23" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>5</v>
+        <v>66</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="C24" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C25" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C27" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
-        <v>17</v>
-      </c>
       <c r="B28" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C28" s="2">
         <v>4</v>
@@ -936,10 +936,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C29" s="2">
         <v>4</v>
@@ -947,53 +947,56 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C30" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C31" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>16</v>
+        <v>24</v>
+      </c>
+      <c r="C32" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>16</v>
@@ -1001,23 +1004,23 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A37" s="17" t="s">
+      <c r="B37" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A38" s="17" t="s">
         <v>57</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
-        <v>64</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>16</v>
@@ -1025,15 +1028,15 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>14</v>
@@ -1041,7 +1044,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>14</v>
@@ -1049,15 +1052,15 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>15</v>
@@ -1065,17 +1068,25 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="16" t="s">
         <v>71</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B46" s="6" t="s">
         <v>72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added a language button to ckeditor.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@230 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="84">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -52,9 +52,6 @@
     <t>EIEOL editor - make glossed texts use CKEditor</t>
   </si>
   <si>
-    <t>CKEditor - Add language plugin http://ckeditor.com/forums/Plugins/Language-Semantics, use our lang and class attributes with it</t>
-  </si>
-  <si>
     <t>When updating glossed texts and glosses, make sure they match so the clickable interface will work</t>
   </si>
   <si>
@@ -277,10 +274,13 @@
     <t>early lesson series often had the bibliography as a section in the 10th lesson.  Later lessons have a bibliography that is essentially a separate page.</t>
   </si>
   <si>
-    <t xml:space="preserve">Add marking foreign words as a push-button feature in CKEditor. </t>
-  </si>
-  <si>
-    <t>Fixed bullet formatting</t>
+    <t>Fix bullet formatting</t>
+  </si>
+  <si>
+    <t>I added italics to the classes</t>
+  </si>
+  <si>
+    <t>CKEditor - Add language button to create a span tag that uses our lang and class attributes with it</t>
   </si>
 </sst>
 </file>
@@ -685,7 +685,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="89.28515625" style="16" customWidth="1"/>
@@ -696,129 +696,140 @@
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="16" t="s">
+        <v>67</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>68</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B4" s="9"/>
       <c r="C4" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D4" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="21" t="s">
+    </row>
+    <row r="5" spans="1:4" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A5" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="8" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="16" t="s">
+      <c r="B7" s="9"/>
+      <c r="C7" s="10" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="16" t="s">
-        <v>7</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="2">
-        <v>1</v>
-      </c>
-    </row>
     <row r="8" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>83</v>
-      </c>
+      <c r="A8" s="8"/>
       <c r="B8" s="9"/>
-      <c r="C8" s="10" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="10"/>
+      <c r="C8" s="10"/>
+    </row>
+    <row r="10" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="19">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
         <v>36</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C11" s="19">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D11" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C12" s="19">
         <v>0</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="B13" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="C13" s="19">
-        <v>0</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
+        <v>1</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="16" t="s">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C17" s="2">
         <v>2</v>
@@ -829,29 +840,29 @@
         <v>61</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C20" s="2">
         <v>2</v>
@@ -859,29 +870,29 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C21" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="16" t="s">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C22" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="B23" s="6" t="s">
         <v>15</v>
@@ -890,45 +901,45 @@
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>66</v>
+        <v>5</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C24" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C25" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C27" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C28" s="2">
         <v>4</v>
@@ -936,7 +947,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B29" s="6" t="s">
         <v>14</v>
@@ -947,48 +958,45 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
+        <v>2</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A31" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="B30" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C30" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
-        <v>2</v>
-      </c>
       <c r="B31" s="6" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C31" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" s="2">
-        <v>5</v>
+        <v>15</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B34" s="6" t="s">
         <v>15</v>
@@ -999,55 +1007,55 @@
         <v>52</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A37" s="17" t="s">
         <v>56</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A38" s="17" t="s">
-        <v>57</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="16" t="s">
+        <v>63</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
@@ -1060,34 +1068,26 @@
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
         <v>71</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1117,13 +1117,13 @@
   <sheetData>
     <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>12</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:4" s="11" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1131,21 +1131,21 @@
         <v>3</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="11" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1153,40 +1153,40 @@
         <v>4</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C7" s="10">
         <v>1</v>
@@ -1194,10 +1194,10 @@
     </row>
     <row r="8" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" s="10">
         <v>0</v>
@@ -1205,24 +1205,24 @@
     </row>
     <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" s="10">
         <v>0</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C10" s="10">
         <v>0</v>
@@ -1230,22 +1230,22 @@
     </row>
     <row r="11" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C11" s="10"/>
       <c r="D11" s="11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" s="10">
         <v>-1</v>
@@ -1256,46 +1256,46 @@
         <v>6</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:4" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C16" s="10">
         <v>0</v>
       </c>
       <c r="D16" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
@@ -1323,42 +1323,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cleaned up Eieol Language plugin
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@231 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="86">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -281,13 +281,19 @@
   </si>
   <si>
     <t>CKEditor - Add language button to create a span tag that uses our lang and class attributes with it</t>
+  </si>
+  <si>
+    <t>Change lesson menus, make Other lessons collapsible.  Move resouces up</t>
+  </si>
+  <si>
+    <t>Output lessons from Admin site, formatted for LaTeX</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -324,6 +330,13 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF00B0F0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="12"/>
       <color rgb="FF00B050"/>
       <name val="Times New Roman"/>
@@ -350,7 +363,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -404,7 +417,26 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -685,7 +717,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D47"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="89.28515625" style="16" customWidth="1"/>
@@ -735,7 +767,7 @@
       <c r="C4" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="28" t="s">
         <v>80</v>
       </c>
     </row>
@@ -749,14 +781,14 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:4" s="24" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="21" t="s">
         <v>83</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="23" t="s">
         <v>79</v>
       </c>
     </row>
@@ -769,67 +801,63 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8"/>
-      <c r="B8" s="9"/>
-      <c r="C8" s="10"/>
-    </row>
-    <row r="10" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C10" s="19">
-        <v>0</v>
-      </c>
+    <row r="8" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B8" s="26"/>
+      <c r="C8" s="27"/>
+    </row>
+    <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="8"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="10"/>
     </row>
     <row r="11" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="16" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C11" s="19">
         <v>0</v>
       </c>
-      <c r="D11" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C12" s="19">
         <v>0</v>
       </c>
       <c r="D12" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="B13" s="18" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="19">
+        <v>0</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="16" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="B16" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
-        <v>60</v>
-      </c>
       <c r="B17" s="6" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C17" s="2">
         <v>2</v>
@@ -837,18 +865,18 @@
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="16" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C18" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="16" t="s">
-        <v>7</v>
+        <v>61</v>
       </c>
       <c r="B19" s="6" t="s">
         <v>14</v>
@@ -857,9 +885,9 @@
         <v>2</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="16" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B20" s="6" t="s">
         <v>14</v>
@@ -870,76 +898,76 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C21" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
-        <v>18</v>
-      </c>
       <c r="B22" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C22" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="16" t="s">
-        <v>65</v>
+        <v>18</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C23" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="16" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C24" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="16" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C25" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="16" t="s">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C26" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A28" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="B27" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C27" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
-        <v>16</v>
-      </c>
       <c r="B28" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C28" s="2">
         <v>4</v>
@@ -947,10 +975,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C29" s="2">
         <v>4</v>
@@ -958,53 +986,56 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="B30" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C30" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C31" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>15</v>
+        <v>23</v>
+      </c>
+      <c r="C32" s="2">
+        <v>5</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="16" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>15</v>
@@ -1012,23 +1043,23 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="B36" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A37" s="17" t="s">
+      <c r="B37" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A38" s="17" t="s">
         <v>56</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="16" t="s">
-        <v>63</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>15</v>
@@ -1036,15 +1067,15 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="B40" s="6" t="s">
         <v>13</v>
@@ -1052,7 +1083,7 @@
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="B41" s="6" t="s">
         <v>13</v>
@@ -1060,15 +1091,15 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B43" s="6" t="s">
         <v>14</v>
@@ -1076,18 +1107,34 @@
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="16" t="s">
         <v>70</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B46" s="6" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="16" t="s">
+        <v>85</v>
+      </c>
+      <c r="B47" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made series menu accordian
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@232 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14955" windowHeight="7305"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14955" windowHeight="7305" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Francis" sheetId="1" r:id="rId1"/>
@@ -293,7 +293,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -311,13 +311,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -325,13 +318,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FF00B050"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF00B0F0"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -363,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -383,17 +369,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -403,40 +402,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -720,7 +686,7 @@
   <dimension ref="A1:D47"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="89.28515625" style="16" customWidth="1"/>
+    <col min="1" max="1" width="89.28515625" style="12" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
@@ -738,7 +704,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="12" t="s">
         <v>67</v>
       </c>
       <c r="B2" s="6" t="s">
@@ -749,7 +715,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="12" t="s">
         <v>75</v>
       </c>
       <c r="B3" s="6" t="s">
@@ -759,93 +725,51 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="D4" s="28" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>78</v>
-      </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="11" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" s="24" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="B6" s="22" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="23" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="10" t="s">
-        <v>79</v>
-      </c>
-    </row>
     <row r="8" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+      <c r="A8" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="B8" s="26"/>
-      <c r="C8" s="27"/>
+      <c r="B8" s="18"/>
+      <c r="C8" s="19"/>
     </row>
     <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="10"/>
     </row>
-    <row r="11" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="16" t="s">
+    <row r="11" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="19">
+      <c r="B11" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C11" s="15">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+    <row r="12" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B12" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="19">
+      <c r="B12" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="15">
         <v>0</v>
       </c>
       <c r="D12" s="7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="20" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+    <row r="13" spans="1:4" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B13" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="19">
+      <c r="B13" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C13" s="15">
         <v>0</v>
       </c>
       <c r="D13" s="7" t="s">
@@ -853,7 +777,7 @@
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="12" t="s">
         <v>1</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -864,7 +788,7 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="12" t="s">
         <v>60</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -875,7 +799,7 @@
       </c>
     </row>
     <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="16" t="s">
+      <c r="A19" s="12" t="s">
         <v>61</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -886,7 +810,7 @@
       </c>
     </row>
     <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -897,7 +821,7 @@
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="16" t="s">
+      <c r="A21" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B21" s="6" t="s">
@@ -908,7 +832,7 @@
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="16" t="s">
+      <c r="A22" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B22" s="6" t="s">
@@ -919,7 +843,7 @@
       </c>
     </row>
     <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="16" t="s">
+      <c r="A23" s="12" t="s">
         <v>18</v>
       </c>
       <c r="B23" s="6" t="s">
@@ -930,7 +854,7 @@
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="12" t="s">
         <v>65</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -941,7 +865,7 @@
       </c>
     </row>
     <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A25" s="16" t="s">
+      <c r="A25" s="12" t="s">
         <v>5</v>
       </c>
       <c r="B25" s="6" t="s">
@@ -952,7 +876,7 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="12" t="s">
         <v>8</v>
       </c>
       <c r="B26" s="6" t="s">
@@ -963,7 +887,7 @@
       </c>
     </row>
     <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A28" s="16" t="s">
+      <c r="A28" s="12" t="s">
         <v>31</v>
       </c>
       <c r="B28" s="6" t="s">
@@ -974,7 +898,7 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="16" t="s">
+      <c r="A29" s="12" t="s">
         <v>16</v>
       </c>
       <c r="B29" s="6" t="s">
@@ -985,7 +909,7 @@
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="16" t="s">
+      <c r="A30" s="12" t="s">
         <v>21</v>
       </c>
       <c r="B30" s="6" t="s">
@@ -996,7 +920,7 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="16" t="s">
+      <c r="A31" s="12" t="s">
         <v>2</v>
       </c>
       <c r="B31" s="6" t="s">
@@ -1007,7 +931,7 @@
       </c>
     </row>
     <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="12" t="s">
         <v>22</v>
       </c>
       <c r="B32" s="6" t="s">
@@ -1018,7 +942,7 @@
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="16" t="s">
+      <c r="A33" s="12" t="s">
         <v>25</v>
       </c>
       <c r="B33" s="6" t="s">
@@ -1026,7 +950,7 @@
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="12" t="s">
         <v>46</v>
       </c>
       <c r="B34" s="6" t="s">
@@ -1034,7 +958,7 @@
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="12" t="s">
         <v>51</v>
       </c>
       <c r="B35" s="6" t="s">
@@ -1042,7 +966,7 @@
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="16" t="s">
+      <c r="A36" s="12" t="s">
         <v>52</v>
       </c>
       <c r="B36" s="6" t="s">
@@ -1050,7 +974,7 @@
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="16" t="s">
+      <c r="A37" s="12" t="s">
         <v>55</v>
       </c>
       <c r="B37" s="6" t="s">
@@ -1058,7 +982,7 @@
       </c>
     </row>
     <row r="38" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A38" s="17" t="s">
+      <c r="A38" s="13" t="s">
         <v>56</v>
       </c>
       <c r="B38" s="6" t="s">
@@ -1066,7 +990,7 @@
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="16" t="s">
+      <c r="A39" s="12" t="s">
         <v>63</v>
       </c>
       <c r="B39" s="6" t="s">
@@ -1074,7 +998,7 @@
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="16" t="s">
+      <c r="A40" s="12" t="s">
         <v>57</v>
       </c>
       <c r="B40" s="6" t="s">
@@ -1082,7 +1006,7 @@
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="16" t="s">
+      <c r="A41" s="12" t="s">
         <v>66</v>
       </c>
       <c r="B41" s="6" t="s">
@@ -1090,7 +1014,7 @@
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="16" t="s">
+      <c r="A42" s="12" t="s">
         <v>58</v>
       </c>
       <c r="B42" s="6" t="s">
@@ -1098,7 +1022,7 @@
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="16" t="s">
+      <c r="A43" s="12" t="s">
         <v>59</v>
       </c>
       <c r="B43" s="6" t="s">
@@ -1106,7 +1030,7 @@
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="16" t="s">
+      <c r="A44" s="12" t="s">
         <v>62</v>
       </c>
       <c r="B44" s="6" t="s">
@@ -1114,7 +1038,7 @@
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="16" t="s">
+      <c r="A45" s="12" t="s">
         <v>64</v>
       </c>
       <c r="B45" s="6" t="s">
@@ -1122,7 +1046,7 @@
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="16" t="s">
+      <c r="A46" s="12" t="s">
         <v>70</v>
       </c>
       <c r="B46" s="6" t="s">
@@ -1130,7 +1054,7 @@
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="16" t="s">
+      <c r="A47" s="12" t="s">
         <v>85</v>
       </c>
       <c r="B47" s="6" t="s">
@@ -1345,13 +1269,47 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="7"/>
-    </row>
-    <row r="19" spans="1:4" s="15" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="12"/>
-      <c r="B19" s="13"/>
-      <c r="C19" s="14"/>
+    <row r="17" spans="1:4" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D17" s="20" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="9"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="11" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20" s="9"/>
+      <c r="C20" s="10" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>

</xml_diff>

<commit_message>
tweaked keep dead languages alive
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@234 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14955" windowHeight="7305" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14955" windowHeight="7305"/>
   </bookViews>
   <sheets>
     <sheet name="Francis" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="86">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -349,7 +349,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -393,15 +393,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -683,7 +674,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="89.28515625" style="12" customWidth="1"/>
@@ -725,225 +716,258 @@
         <v>69</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="7" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="17" t="s">
-        <v>84</v>
-      </c>
-      <c r="B8" s="18"/>
-      <c r="C8" s="19"/>
-    </row>
-    <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="10"/>
-    </row>
-    <row r="11" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="12" t="s">
+    <row r="4" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10"/>
+    </row>
+    <row r="6" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11" s="15">
+      <c r="B6" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="15">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7" s="15">
+        <v>0</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A8" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="15">
+        <v>0</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="15">
-        <v>0</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B13" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="15">
-        <v>0</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>39</v>
+        <v>60</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A14" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="2">
+        <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="12" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C17" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>60</v>
+        <v>18</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C18" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C19" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C20" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B21" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C21" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C23" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C24" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="C25" s="2">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C26" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B28" s="6" t="s">
         <v>15</v>
-      </c>
-      <c r="C28" s="2">
-        <v>4</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>16</v>
+        <v>46</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="2">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" s="2">
-        <v>4</v>
+        <v>15</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C31" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="12" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C32" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A33" s="12" t="s">
-        <v>25</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="75" x14ac:dyDescent="0.25">
+      <c r="A33" s="13" t="s">
+        <v>56</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>15</v>
@@ -951,113 +975,73 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>46</v>
+        <v>63</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A38" s="13" t="s">
-        <v>56</v>
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="12" t="s">
+        <v>59</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>13</v>
+        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>58</v>
+        <v>85</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A43" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A44" s="12" t="s">
-        <v>62</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
-        <v>64</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A46" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B46" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A47" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="B47" s="6" t="s">
         <v>17</v>
       </c>
     </row>
@@ -1277,7 +1261,7 @@
       <c r="C17" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="17" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1308,6 +1292,17 @@
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="10" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="8" t="s">
+        <v>84</v>
+      </c>
+      <c r="B21" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="10" t="s">
         <v>79</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Changed Parts of Speech and Analysis to be unique per language.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@236 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -256,9 +256,6 @@
     <t>Decide where to put links to the new LRC site on the center site</t>
   </si>
   <si>
-    <t>EIEOL - attach parts of speech and analysis to languages - use features file to load new one.  Sweep glosses to use new ones, change language editor, change pulldowns in gloss editor.  Add comment box to each pos and analysis.  Remove old POS and analysis editors</t>
-  </si>
-  <si>
     <t>umlauts are adding a space after the letter in some browsers.  See https://lrc.la.utexas.edu/eieol_lesson/7?id=929 - Grammars/2nd paragraph/1st word.  Browser specific?</t>
   </si>
   <si>
@@ -287,6 +284,9 @@
   </si>
   <si>
     <t>Output lessons from Admin site, formatted for LaTeX</t>
+  </si>
+  <si>
+    <t>EIEOL - attach parts of speech and analysis to languages.  Sweep elements to use new ones, change language editor, change pulldowns in gloss editor.  Remove old POS and analysis editors</t>
   </si>
 </sst>
 </file>
@@ -705,9 +705,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>17</v>
@@ -1039,7 +1039,7 @@
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="12" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B42" s="6" t="s">
         <v>17</v>
@@ -1214,7 +1214,7 @@
         <v>13</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="14" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1225,18 +1225,18 @@
         <v>13</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:4" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B15" s="9" t="s">
         <v>13</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
@@ -1255,55 +1255,55 @@
     </row>
     <row r="17" spans="1:4" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B17" s="9"/>
       <c r="C17" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="D17" s="17" t="s">
         <v>79</v>
-      </c>
-      <c r="D17" s="17" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:4" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B18" s="9"/>
       <c r="C18" s="10"/>
       <c r="D18" s="11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="19" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B19" s="9" t="s">
         <v>14</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B20" s="9"/>
       <c r="C20" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B21" s="9" t="s">
         <v>13</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Fixed bug.  Lesson text wasn't being displayed on editor since I installed ckeditor.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@239 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14955" windowHeight="7305"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13200" windowHeight="7305"/>
   </bookViews>
   <sheets>
     <sheet name="Francis" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="87">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -287,13 +287,16 @@
   </si>
   <si>
     <t>EIEOL - attach parts of speech and analysis to languages.  Sweep elements to use new ones, change language editor, change pulldowns in gloss editor.  Remove old POS and analysis editors</t>
+  </si>
+  <si>
+    <t>would it be possible (and would it refine the output, rather than making it balloon) to have searches with multiple items?  What I mean is, if I start typing "3", I'll get a lot of PoSs with "3rd person singular" and "3rd person plural".  In fact there are so many options that the ones with "singular" do not appear on the screen, since alphabetization pushes them below "plural".  To get the "singular" options, I have to type the *entire* PoS in full up to the "s" of singular before these options begin to appear.  Would it be possible to type instead "3 p s" and have the list refine to options with the 1st element beginning with "3", the second with "p", the third with "s"?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -328,6 +331,12 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -349,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -394,6 +403,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -674,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="89.28515625" style="12" customWidth="1"/>
@@ -1043,6 +1055,11 @@
       </c>
       <c r="B42" s="6" t="s">
         <v>17</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="18" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed user page. Renamed delete button to clear.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@242 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="87">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -686,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="89.28515625" style="12" customWidth="1"/>
@@ -987,15 +987,15 @@
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="12" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="B35" s="6" t="s">
         <v>13</v>
@@ -1003,7 +1003,7 @@
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="12" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="B36" s="6" t="s">
         <v>13</v>
@@ -1011,15 +1011,15 @@
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="12" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B38" s="6" t="s">
         <v>14</v>
@@ -1027,38 +1027,30 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="12" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="12" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>17</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="12" t="s">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A42" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="B42" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="43" spans="1:2" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="18" t="s">
+    <row r="42" spans="1:2" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="18" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1323,6 +1315,17 @@
         <v>78</v>
       </c>
     </row>
+    <row r="22" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>78</v>
+      </c>
+    </row>
     <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Built EIEOL text pages.  Also a few cleanups of links and images
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@252 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="89">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -136,9 +136,6 @@
     <t>DOI - Digital Object Identifier - register with DOI sites.</t>
   </si>
   <si>
-    <t>Review links and toolbars with users</t>
-  </si>
-  <si>
     <t>remove load controller, load views, references in routes.php and app/storage/data_load/</t>
   </si>
   <si>
@@ -166,9 +163,6 @@
     <t>TEST, TEST, TEST</t>
   </si>
   <si>
-    <t>Move content from Old site to center site.</t>
-  </si>
-  <si>
     <t>Use EIDs instead of our own logons?</t>
   </si>
   <si>
@@ -235,12 +229,6 @@
     <t>In lesson editor, need a way of flagging glosses and textareas that have mistakes and add comment so another admin can fix.  Admin comments (only admin can edit) Author comments.</t>
   </si>
   <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>A3</t>
-  </si>
-  <si>
     <t xml:space="preserve">In the editor, add links to instructional pages that Todd will create </t>
   </si>
   <si>
@@ -250,12 +238,6 @@
     <t>Design a Unicode test page.  Give them a bunch of text and a screenshot of what it should look like.</t>
   </si>
   <si>
-    <t>Decide what links to put in the menus on the new LRC site</t>
-  </si>
-  <si>
-    <t>Decide where to put links to the new LRC site on the center site</t>
-  </si>
-  <si>
     <t>umlauts are adding a space after the letter in some browsers.  See https://lrc.la.utexas.edu/eieol_lesson/7?id=929 - Grammars/2nd paragraph/1st word.  Browser specific?</t>
   </si>
   <si>
@@ -290,13 +272,37 @@
   </si>
   <si>
     <t>would it be possible (and would it refine the output, rather than making it balloon) to have searches with multiple items?  What I mean is, if I start typing "3", I'll get a lot of PoSs with "3rd person singular" and "3rd person plural".  In fact there are so many options that the ones with "singular" do not appear on the screen, since alphabetization pushes them below "plural".  To get the "singular" options, I have to type the *entire* PoS in full up to the "s" of singular before these options begin to appear.  Would it be possible to type instead "3 p s" and have the list refine to options with the 1st element beginning with "3", the second with "p", the third with "s"?</t>
+  </si>
+  <si>
+    <t>Done 1/7/2016</t>
+  </si>
+  <si>
+    <t>EIEOL - Remove references to Unicode</t>
+  </si>
+  <si>
+    <t>Build a preview page to view a lesson before publishing it</t>
+  </si>
+  <si>
+    <t>Accessiblity testing</t>
+  </si>
+  <si>
+    <t>EIEOL print on demand - Research options</t>
+  </si>
+  <si>
+    <t>Build Text pages from EIEOL content</t>
+  </si>
+  <si>
+    <t>with Francis - Decide where to put links to the new LRC site on the center site and what links to put in the menus on the new LRC site</t>
+  </si>
+  <si>
+    <t>with Todd - Decide where to put links to the new LRC site on the center site and what links to put in the menus on the new LRC site</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,12 +314,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -333,7 +333,6 @@
     </font>
     <font>
       <sz val="12"/>
-      <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
@@ -378,33 +377,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="10" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -686,10 +689,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="89.28515625" style="12" customWidth="1"/>
+    <col min="1" max="1" width="116.5703125" style="11" customWidth="1"/>
     <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
@@ -706,97 +709,114 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="12" t="s">
+    <row r="2" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>85</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B4" s="18" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="10">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="9">
+        <v>1</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="9">
+        <v>1</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="10"/>
-    </row>
-    <row r="6" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="B6" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="15">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="15">
-        <v>0</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" s="16" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" s="15">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="12" t="s">
-        <v>1</v>
+      <c r="C11" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>59</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C12" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A13" s="12" t="s">
-        <v>60</v>
+    <row r="13" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>7</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="30" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
-        <v>61</v>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>9</v>
       </c>
       <c r="B14" s="6" t="s">
         <v>14</v>
@@ -805,31 +825,31 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
-        <v>7</v>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>0</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C15" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
-        <v>9</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>18</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C16" s="2">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
-        <v>0</v>
+      <c r="A17" s="11" t="s">
+        <v>63</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>15</v>
@@ -839,219 +859,197 @@
       </c>
     </row>
     <row r="18" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
-        <v>18</v>
+      <c r="A18" s="11" t="s">
+        <v>5</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="C18" s="2">
         <v>3</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="12" t="s">
-        <v>65</v>
+      <c r="A19" s="11" t="s">
+        <v>8</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>5</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C20" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
-        <v>8</v>
+    <row r="21" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>31</v>
       </c>
       <c r="B21" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="C21" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="C23" s="2">
         <v>4</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="12" t="s">
-        <v>16</v>
+      <c r="A24" s="11" t="s">
+        <v>2</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C24" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="12" t="s">
-        <v>21</v>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="30" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
+        <v>22</v>
       </c>
       <c r="B25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="B27" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C25" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="B26" s="6" t="s">
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>53</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="60" x14ac:dyDescent="0.25">
+      <c r="A31" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B35" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C26" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C27" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="B28" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="12" t="s">
-        <v>46</v>
-      </c>
-      <c r="B29" s="6" t="s">
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B36" s="6" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="12" t="s">
-        <v>51</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="B32" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="75" x14ac:dyDescent="0.25">
-      <c r="A33" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="B33" s="6" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A34" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A35" s="12" t="s">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="B35" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A36" s="12" t="s">
-        <v>58</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A37" s="12" t="s">
-        <v>59</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A38" s="12" t="s">
-        <v>62</v>
-      </c>
       <c r="B38" s="6" t="s">
-        <v>14</v>
+        <v>67</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A39" s="12" t="s">
-        <v>64</v>
+      <c r="A39" s="11" t="s">
+        <v>78</v>
       </c>
       <c r="B39" s="6" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A40" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A41" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="B41" s="6" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="18" t="s">
-        <v>86</v>
+    <row r="40" spans="1:2" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
+        <v>80</v>
       </c>
     </row>
   </sheetData>
@@ -1090,243 +1088,286 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="11" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8" t="s">
+    <row r="2" spans="1:4" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="10" t="s">
+      <c r="B2" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="11" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+    <row r="3" spans="1:4" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="10" t="s">
+      <c r="B3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="8" t="s">
+    <row r="4" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="10" t="s">
+      <c r="B4" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="10" t="s">
+    <row r="5" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="10" t="s">
+      <c r="B6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="9" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="8" t="s">
+    <row r="7" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C7" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="9">
+        <v>0</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="9"/>
+      <c r="D11" s="10" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C12" s="9">
+        <v>-1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" s="10" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
+      <c r="A15" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C16" s="9">
+        <v>0</v>
+      </c>
+      <c r="D16" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C7" s="10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" s="10">
-        <v>0</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
-        <v>40</v>
-      </c>
-      <c r="B10" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10" s="10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="11" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C12" s="10">
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" s="11" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" s="11" customFormat="1" ht="45" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
+    </row>
+    <row r="17" spans="1:4" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="B17" s="8"/>
+      <c r="C17" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="D17" s="13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" s="8"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B16" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C16" s="10">
-        <v>0</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" s="11" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
+    </row>
+    <row r="19" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="7" t="s">
         <v>76</v>
       </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="D17" s="17" t="s">
+      <c r="B19" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="B20" s="8"/>
+      <c r="C20" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C21" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C23" s="9" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+      <c r="A24" s="7" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" s="11" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="11" t="s">
+      <c r="B24" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="9" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="19" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" s="9"/>
-      <c r="C20" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="8" t="s">
+    <row r="25" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
         <v>83</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" s="11" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="B22" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="B25" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" s="17" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -1341,47 +1382,43 @@
     <col min="1" max="1" width="102.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>45</v>
+    <row r="3" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>74</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>73</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Redid sort to do more work up front.  But this broke the handling multiple characters.
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@260 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="13200" windowHeight="7305" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13200" windowHeight="7305"/>
   </bookViews>
   <sheets>
     <sheet name="Francis" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="95">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -308,6 +308,12 @@
   </si>
   <si>
     <t>Done 1/25/2016</t>
+  </si>
+  <si>
+    <t>Allow users to change their own password</t>
+  </si>
+  <si>
+    <t>Expand class and attribute options on language page to allow multiple languages.  Useful for hittite.  Expand language tagging button on lesson editor to handle multiple language.</t>
   </si>
 </sst>
 </file>
@@ -701,7 +707,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D38"/>
+  <dimension ref="A1:D40"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="116.5703125" style="11" customWidth="1"/>
@@ -1040,6 +1046,16 @@
     <row r="38" spans="1:2" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="14" t="s">
         <v>80</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="11" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="11" t="s">
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed load code.  Don't need it anymore, data was loaded over a year ago and hasn't changed
git-svn-id: svn+ssh://source.la.utexas.edu/repos/lrc-site/trunk@272 98d3ac28-6462-4f9b-a335-089c6823c7e4
</commit_message>
<xml_diff>
--- a/Documentation/LRC Backlog.xlsx
+++ b/Documentation/LRC Backlog.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="6" rupBuild="26929"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr autoCompressPictures="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fmcgrath\workspace\lrc-site\Documentation\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="25600" windowHeight="16060"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25605" windowHeight="16065"/>
   </bookViews>
   <sheets>
     <sheet name="Francis" sheetId="1" r:id="rId1"/>
@@ -13,18 +18,18 @@
   </sheets>
   <calcPr calcId="140001" concurrentCalc="0"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
       <mx:ArchID Flags="2"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="110">
   <si>
     <t>Export words that have Tolkien in their gloss to another language</t>
   </si>
@@ -351,6 +356,9 @@
   </si>
   <si>
     <t>This would allow the text box to focus on lesson content rather than page formatting</t>
+  </si>
+  <si>
+    <t>Done 6/6/2016</t>
   </si>
 </sst>
 </file>
@@ -736,7 +744,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns="" xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -744,16 +752,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D43"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+  <dimension ref="A1:D41"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="116.5" style="11" customWidth="1"/>
-    <col min="2" max="2" width="18.1640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="32.83203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="116.42578125" style="11" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="32.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="5" customFormat="1">
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -764,95 +772,92 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="10" customFormat="1">
-      <c r="A2" s="10" t="s">
-        <v>88</v>
-      </c>
-      <c r="B2" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="C2" s="10">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" s="10" customFormat="1">
-      <c r="A3" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="9">
+    <row r="2" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="9">
         <v>1</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" s="10" customFormat="1">
-      <c r="A4" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B4" s="8" t="s">
+      <c r="D2" s="10" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="9">
-        <v>1</v>
-      </c>
-      <c r="D4" s="10" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4">
+      <c r="C6" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>58</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="11" t="s">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="9" spans="1:4">
+      <c r="D8" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="11" t="s">
-        <v>58</v>
+        <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C9" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="28">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="11" t="s">
-        <v>59</v>
+        <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
         <v>14</v>
       </c>
       <c r="C10" s="2">
-        <v>2</v>
-      </c>
-      <c r="D10" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="11" t="s">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C11" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="11" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>14</v>
@@ -861,144 +866,144 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="11" t="s">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="B13" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C13" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="6" t="s">
+    <row r="17" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C17" s="2">
+        <v>4</v>
+      </c>
+      <c r="D17" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C18" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="C14" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="11" t="s">
-        <v>63</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4">
-      <c r="A16" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C16" s="2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4">
-      <c r="A17" s="11" t="s">
-        <v>8</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="28">
-      <c r="A19" s="11" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="C19" s="2">
         <v>4</v>
       </c>
-      <c r="D19" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4">
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="11" t="s">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C20" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="11" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>14</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C22" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="28">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="11" t="s">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C23" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:4">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="11" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="B24" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C24" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C25" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="11" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B26" s="6" t="s">
         <v>15</v>
@@ -1007,196 +1012,174 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:4">
-      <c r="A27" s="11" t="s">
-        <v>50</v>
+    <row r="27" spans="1:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="A27" s="12" t="s">
+        <v>54</v>
       </c>
       <c r="B27" s="6" t="s">
         <v>15</v>
       </c>
       <c r="C27" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="11" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C28" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="42">
-      <c r="A29" s="12" t="s">
-        <v>54</v>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
+        <v>64</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C29" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D30" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C31" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:4">
-      <c r="A30" s="11" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" s="2">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4">
-      <c r="A31" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C31" s="2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="11" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="D32" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4">
+        <v>14</v>
+      </c>
+      <c r="C32" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B33" s="6" t="s">
         <v>17</v>
       </c>
       <c r="C33" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="11" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C34" s="2">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4">
+        <v>67</v>
+      </c>
+      <c r="D34" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="11" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="B35" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C35" s="2">
+        <v>1</v>
+      </c>
+      <c r="D35" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="14" t="s">
+        <v>80</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C36" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C37" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A38" s="11" t="s">
+        <v>94</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C35" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4">
-      <c r="A36" s="11" t="s">
-        <v>66</v>
-      </c>
-      <c r="B36" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D36" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4">
-      <c r="A37" s="11" t="s">
-        <v>78</v>
-      </c>
-      <c r="B37" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C37" s="2">
+      <c r="C38" s="2">
         <v>1</v>
       </c>
-      <c r="D37" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" ht="89.25" customHeight="1">
-      <c r="A38" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="B38" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C38" s="2">
+      <c r="D38" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A39" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C39" s="2">
+        <v>1</v>
+      </c>
+      <c r="D39" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+      <c r="A40" s="11" t="s">
+        <v>106</v>
+      </c>
+      <c r="C40" s="2">
         <v>2</v>
       </c>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="B39" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C39" s="2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" ht="28">
-      <c r="A40" s="11" t="s">
-        <v>94</v>
-      </c>
-      <c r="B40" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C40" s="2">
-        <v>1</v>
-      </c>
       <c r="D40" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" ht="28">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="11" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="C41" s="2">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D41" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4">
-      <c r="A42" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="C42" s="2">
-        <v>2</v>
-      </c>
-      <c r="D42" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4">
-      <c r="A43" s="11" t="s">
-        <v>107</v>
-      </c>
-      <c r="C43" s="2">
-        <v>2</v>
-      </c>
-      <c r="D43" t="s">
         <v>108</v>
       </c>
     </row>
@@ -1216,16 +1199,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="88.5" style="1" customWidth="1"/>
-    <col min="2" max="2" width="18.1640625" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="88.42578125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="18.140625" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.28515625" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="5" customFormat="1">
+    <row r="1" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -1236,7 +1219,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="10" customFormat="1" ht="18.75" customHeight="1">
+    <row r="2" spans="1:4" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
         <v>3</v>
       </c>
@@ -1247,7 +1230,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="3" spans="1:4" s="10" customFormat="1" ht="18.75" customHeight="1">
+    <row r="3" spans="1:4" s="10" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>20</v>
       </c>
@@ -1258,7 +1241,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="4" spans="1:4" s="10" customFormat="1">
+    <row r="4" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>4</v>
       </c>
@@ -1269,7 +1252,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:4" s="10" customFormat="1">
+    <row r="5" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>42</v>
       </c>
@@ -1280,7 +1263,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="6" spans="1:4" s="10" customFormat="1">
+    <row r="6" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7" t="s">
         <v>29</v>
       </c>
@@ -1291,7 +1274,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="7" spans="1:4" s="10" customFormat="1">
+    <row r="7" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>45</v>
       </c>
@@ -1302,7 +1285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:4" s="10" customFormat="1">
+    <row r="8" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>30</v>
       </c>
@@ -1313,7 +1296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:4" s="10" customFormat="1">
+    <row r="9" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>40</v>
       </c>
@@ -1327,7 +1310,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="10" spans="1:4" s="10" customFormat="1">
+    <row r="10" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>39</v>
       </c>
@@ -1338,7 +1321,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:4" s="10" customFormat="1">
+    <row r="11" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>24</v>
       </c>
@@ -1350,7 +1333,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:4" s="10" customFormat="1">
+    <row r="12" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>46</v>
       </c>
@@ -1361,7 +1344,7 @@
         <v>-1</v>
       </c>
     </row>
-    <row r="13" spans="1:4" s="10" customFormat="1" ht="14.25" customHeight="1">
+    <row r="13" spans="1:4" s="10" customFormat="1" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>6</v>
       </c>
@@ -1372,7 +1355,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:4" s="10" customFormat="1">
+    <row r="14" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>52</v>
       </c>
@@ -1383,7 +1366,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:4" s="10" customFormat="1" ht="28">
+    <row r="15" spans="1:4" s="10" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>69</v>
       </c>
@@ -1394,7 +1377,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:4" s="10" customFormat="1">
+    <row r="16" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>51</v>
       </c>
@@ -1408,7 +1391,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:4" s="10" customFormat="1" ht="15">
+    <row r="17" spans="1:4" s="10" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>70</v>
       </c>
@@ -1420,7 +1403,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:4" s="10" customFormat="1">
+    <row r="18" spans="1:4" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>71</v>
       </c>
@@ -1430,7 +1413,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="19" spans="1:4" s="10" customFormat="1">
+    <row r="19" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>76</v>
       </c>
@@ -1441,7 +1424,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:4" s="10" customFormat="1">
+    <row r="20" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>74</v>
       </c>
@@ -1450,7 +1433,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="21" spans="1:4" s="10" customFormat="1">
+    <row r="21" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>77</v>
       </c>
@@ -1461,7 +1444,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="1:4" s="10" customFormat="1">
+    <row r="22" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>61</v>
       </c>
@@ -1472,7 +1455,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:4" s="10" customFormat="1" ht="28">
+    <row r="23" spans="1:4" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>65</v>
       </c>
@@ -1483,7 +1466,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:4" s="10" customFormat="1" ht="28">
+    <row r="24" spans="1:4" s="10" customFormat="1" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>79</v>
       </c>
@@ -1494,7 +1477,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="1:4" s="16" customFormat="1">
+    <row r="25" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="15" t="s">
         <v>83</v>
       </c>
@@ -1505,7 +1488,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:4" s="16" customFormat="1">
+    <row r="26" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="15" t="s">
         <v>86</v>
       </c>
@@ -1516,7 +1499,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="27" spans="1:4" s="16" customFormat="1">
+    <row r="27" spans="1:4" s="16" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
         <v>84</v>
       </c>
@@ -1527,7 +1510,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:4" s="10" customFormat="1">
+    <row r="28" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>85</v>
       </c>
@@ -1536,6 +1519,31 @@
       </c>
       <c r="C28" s="18" t="s">
         <v>90</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" s="10" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="9">
+        <v>1</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1552,42 +1560,42 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14" x14ac:dyDescent="0"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="102.5" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="102.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" s="10" customFormat="1">
+    <row r="1" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="2" spans="1:1" s="10" customFormat="1">
+    <row r="2" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" spans="1:1" s="10" customFormat="1">
+    <row r="3" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:1" s="10" customFormat="1">
+    <row r="4" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:1" s="10" customFormat="1">
+    <row r="5" spans="1:1" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="7" spans="1:1">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>34</v>
       </c>

</xml_diff>